<commit_message>
New execise of 6_ : PEATONES
</commit_message>
<xml_diff>
--- a/Data/nuevo.xlsx
+++ b/Data/nuevo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
new pptx and more
</commit_message>
<xml_diff>
--- a/Data/nuevo.xlsx
+++ b/Data/nuevo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
           <t>Población</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Menor_edad</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -459,6 +464,9 @@
           <t>Madrid</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -474,6 +482,9 @@
           <t>Sevilla</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -489,6 +500,9 @@
           <t>Valencia</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -504,6 +518,9 @@
           <t>Segovia</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -519,6 +536,9 @@
           <t>Madrid</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -534,18 +554,8 @@
           <t>Madrid</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Amelia</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Toledo</t>
-        </is>
+      <c r="D7" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>